<commit_message>
Update freshwater catch notes
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7480D243-972A-45A9-B176-D78F873E10AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53ED5955-FA3E-40C7-81E7-C6EA309863FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
@@ -176,9 +176,6 @@
     <t>No creel survey in 2018</t>
   </si>
   <si>
-    <t>FSC data source</t>
-  </si>
-  <si>
     <t>Robichaud &amp; English 2012, Tables 11, 13</t>
   </si>
   <si>
@@ -204,6 +201,9 @@
   </si>
   <si>
     <t>General source</t>
+  </si>
+  <si>
+    <t>FN FSC data source</t>
   </si>
 </sst>
 </file>
@@ -804,7 +804,7 @@
         <v>12</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q1" s="2" t="s">
         <v>44</v>
@@ -813,7 +813,7 @@
         <v>32</v>
       </c>
       <c r="S1" s="18" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="T1" s="18" t="s">
         <v>35</v>
@@ -908,7 +908,7 @@
       </c>
       <c r="R2" s="7"/>
       <c r="S2" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T2" s="7"/>
       <c r="U2" s="7"/>
@@ -988,7 +988,7 @@
       </c>
       <c r="R3" s="5"/>
       <c r="S3" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T3" s="5"/>
       <c r="U3" s="5"/>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="R4" s="5"/>
       <c r="S4" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T4" s="5"/>
       <c r="U4" s="5"/>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="R5" s="5"/>
       <c r="S5" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T5" s="5"/>
       <c r="U5" s="5"/>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="R6" s="5"/>
       <c r="S6" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T6" s="5"/>
       <c r="U6" s="5"/>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="R7" s="5"/>
       <c r="S7" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T7" s="5"/>
       <c r="U7" s="5"/>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="R8" s="5"/>
       <c r="S8" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T8" s="5"/>
       <c r="U8" s="5"/>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="R9" s="5"/>
       <c r="S9" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T9" s="5"/>
       <c r="U9" s="5"/>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="R10" s="5"/>
       <c r="S10" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T10" s="5"/>
       <c r="U10" s="5"/>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="R11" s="5"/>
       <c r="S11" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T11" s="5"/>
       <c r="U11" s="5"/>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="R12" s="5"/>
       <c r="S12" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T12" s="5"/>
       <c r="U12" s="5"/>
@@ -1795,7 +1795,7 @@
       </c>
       <c r="R13" s="5"/>
       <c r="S13" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T13" s="5"/>
       <c r="U13" s="5"/>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="R14" s="5"/>
       <c r="S14" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T14" s="5"/>
       <c r="U14" s="5"/>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="R15" s="5"/>
       <c r="S15" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T15" s="5"/>
       <c r="U15" s="5"/>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="R16" s="5"/>
       <c r="S16" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T16" s="5"/>
       <c r="U16" s="5"/>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="R17" s="5"/>
       <c r="S17" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T17" s="5"/>
       <c r="U17" s="5"/>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="R18" s="5"/>
       <c r="S18" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T18" s="5"/>
       <c r="U18" s="5"/>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="R19" s="5"/>
       <c r="S19" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T19" s="5"/>
       <c r="U19" s="5"/>
@@ -2359,7 +2359,7 @@
       <c r="Q20" s="30"/>
       <c r="R20" s="5"/>
       <c r="S20" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T20" s="5"/>
       <c r="U20" s="5"/>
@@ -2436,7 +2436,7 @@
       <c r="Q21" s="30"/>
       <c r="R21" s="5"/>
       <c r="S21" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T21" s="5"/>
       <c r="U21" s="5"/>
@@ -2513,7 +2513,7 @@
       <c r="Q22" s="30"/>
       <c r="R22" s="5"/>
       <c r="S22" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T22" s="5"/>
       <c r="U22" s="5"/>
@@ -2590,7 +2590,7 @@
       <c r="Q23" s="30"/>
       <c r="R23" s="5"/>
       <c r="S23" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T23" s="5"/>
       <c r="U23" s="5"/>
@@ -2667,7 +2667,7 @@
       <c r="Q24" s="30"/>
       <c r="R24" s="5"/>
       <c r="S24" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T24" s="5"/>
       <c r="U24" s="5"/>
@@ -2747,7 +2747,7 @@
         <v>33</v>
       </c>
       <c r="S25" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T25" s="5"/>
       <c r="U25" s="5"/>
@@ -2836,7 +2836,7 @@
         <v>33</v>
       </c>
       <c r="S26" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T26" s="5"/>
       <c r="U26" s="5"/>
@@ -2913,7 +2913,7 @@
       <c r="Q27" s="30"/>
       <c r="R27" s="5"/>
       <c r="S27" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T27" s="5"/>
       <c r="U27" s="5"/>
@@ -2990,7 +2990,7 @@
       <c r="Q28" s="30"/>
       <c r="R28" s="5"/>
       <c r="S28" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T28" s="5"/>
       <c r="U28" s="5"/>
@@ -3067,7 +3067,7 @@
       <c r="Q29" s="30"/>
       <c r="R29" s="5"/>
       <c r="S29" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T29" s="5"/>
       <c r="U29" s="5"/>
@@ -3145,7 +3145,7 @@
       <c r="Q30" s="30"/>
       <c r="R30" s="5"/>
       <c r="S30" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T30" s="5"/>
       <c r="U30" s="5"/>
@@ -3222,7 +3222,7 @@
       <c r="Q31" s="30"/>
       <c r="R31" s="5"/>
       <c r="S31" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T31" s="5"/>
       <c r="U31" s="5"/>
@@ -3299,7 +3299,7 @@
       <c r="Q32" s="30"/>
       <c r="R32" s="5"/>
       <c r="S32" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T32" s="5"/>
       <c r="U32" s="5"/>
@@ -3377,11 +3377,11 @@
         <v>29</v>
       </c>
       <c r="Q33" s="33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R33" s="5"/>
       <c r="S33" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T33" s="5" t="s">
         <v>34</v>
@@ -3459,11 +3459,11 @@
         <v>29</v>
       </c>
       <c r="Q34" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="R34" s="5"/>
       <c r="S34" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T34" s="5" t="s">
         <v>34</v>
@@ -3553,13 +3553,13 @@
         <v>29</v>
       </c>
       <c r="Q35" s="29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="R35" s="5" t="s">
         <v>33</v>
       </c>
       <c r="S35" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T35" s="5" t="s">
         <v>34</v>
@@ -3649,13 +3649,13 @@
         <v>29</v>
       </c>
       <c r="Q36" s="33" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="R36" s="5" t="s">
         <v>33</v>
       </c>
       <c r="S36" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T36" s="5" t="s">
         <v>34</v>
@@ -3745,13 +3745,13 @@
         <v>29</v>
       </c>
       <c r="Q37" s="33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="R37" s="5" t="s">
         <v>33</v>
       </c>
       <c r="S37" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T37" s="5" t="s">
         <v>34</v>
@@ -3841,13 +3841,13 @@
         <v>29</v>
       </c>
       <c r="Q38" s="33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R38" s="5" t="s">
         <v>33</v>
       </c>
       <c r="S38" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T38" s="5" t="s">
         <v>34</v>
@@ -3937,13 +3937,13 @@
         <v>29</v>
       </c>
       <c r="Q39" s="33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R39" s="5" t="s">
         <v>33</v>
       </c>
       <c r="S39" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T39" s="5" t="s">
         <v>34</v>
@@ -4039,7 +4039,7 @@
         <v>33</v>
       </c>
       <c r="S40" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T40" s="5" t="s">
         <v>34</v>
@@ -4133,7 +4133,7 @@
         <v>45</v>
       </c>
       <c r="S41" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T41" s="5"/>
       <c r="U41" s="5"/>
@@ -4227,7 +4227,7 @@
         <v>33</v>
       </c>
       <c r="S42" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T42" s="5"/>
       <c r="U42" s="5"/>
@@ -4321,7 +4321,7 @@
         <v>33</v>
       </c>
       <c r="S43" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T43" s="5"/>
       <c r="U43" s="5"/>
@@ -4412,7 +4412,7 @@
         <v>33</v>
       </c>
       <c r="S44" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T44" s="5"/>
       <c r="U44" s="5"/>
@@ -4503,7 +4503,7 @@
         <v>33</v>
       </c>
       <c r="S45" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T45" s="5"/>
       <c r="U45" s="5"/>
@@ -4594,7 +4594,7 @@
         <v>33</v>
       </c>
       <c r="S46" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T46" s="5"/>
       <c r="U46" s="5"/>
@@ -4685,7 +4685,7 @@
         <v>33</v>
       </c>
       <c r="S47" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T47" s="5"/>
       <c r="U47" s="5"/>
@@ -4768,7 +4768,7 @@
         <v>33</v>
       </c>
       <c r="S48" s="34" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="T48" s="5"/>
       <c r="U48" s="5"/>

</xml_diff>